<commit_message>
Updated The Multiple Contact Deatils Extraction And Oprational Status Logic
</commit_message>
<xml_diff>
--- a/template/Formate_for_genral.xlsx
+++ b/template/Formate_for_genral.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nmr71\OneDrive\Desktop\format\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\google_maps_scraper\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{925522CD-5A5E-46DA-8140-61F2BB2179FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B2BCC2D-828B-4609-B988-6BB4EE068B05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Sr. no.</t>
   </si>
@@ -82,6 +82,21 @@
   </si>
   <si>
     <t xml:space="preserve">Toll free number </t>
+  </si>
+  <si>
+    <t>Business Status</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Rating</t>
+  </si>
+  <si>
+    <t>Reviews Count</t>
+  </si>
+  <si>
+    <t>Scraping Status</t>
   </si>
 </sst>
 </file>
@@ -408,7 +423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:X2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.21875" bestFit="1" customWidth="1"/>
@@ -431,7 +446,7 @@
     <col min="18" max="18" width="11.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -489,8 +504,23 @@
       <c r="S1" s="2" t="s">
         <v>14</v>
       </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" t="s">
+        <v>23</v>
+      </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>

</xml_diff>